<commit_message>
Add AMLC adverse media source
</commit_message>
<xml_diff>
--- a/data/rules/mediaMapping.xlsx
+++ b/data/rules/mediaMapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hajibashi.Saba\Desktop\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2962190-092E-4F94-B8A2-904F960D52DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3799DA64-844C-42B3-9240-0CB325E69628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="91">
   <si>
     <t>Field</t>
   </si>
@@ -242,6 +242,57 @@
   </si>
   <si>
     <t>date.originalValue</t>
+  </si>
+  <si>
+    <t>AMLC_NEWS_AND_ANNOUNCEMENTS TYPE</t>
+  </si>
+  <si>
+    <t>AMLC_NEWS_AND_ANNOUNCEMENTS</t>
+  </si>
+  <si>
+    <t>"AMLC_NEWS_AND_ANNOUNCEMENTS"</t>
+  </si>
+  <si>
+    <t>"AMLC"</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>content</t>
+  </si>
+  <si>
+    <t>publicationDate</t>
+  </si>
+  <si>
+    <t>author</t>
+  </si>
+  <si>
+    <t>"en"</t>
+  </si>
+  <si>
+    <t>list_expand</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>constant*constant*constant</t>
+  </si>
+  <si>
+    <t>"IMAGE"*"IMAGE"*"PDF"</t>
+  </si>
+  <si>
+    <t>list_expand*list_expand*list_expand</t>
+  </si>
+  <si>
+    <t>imageUrl*additionalImageUrls*pdfUrls</t>
   </si>
 </sst>
 </file>
@@ -285,7 +336,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -295,6 +346,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -508,7 +565,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="17.25" style="3" customWidth="1"/>
@@ -517,9 +574,11 @@
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="39.58203125" customWidth="1"/>
     <col min="6" max="6" width="34" customWidth="1"/>
+    <col min="7" max="7" width="17.58203125" customWidth="1"/>
+    <col min="8" max="8" width="24.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="10.65" customHeight="1">
+    <row r="1" spans="1:8" ht="10.65" customHeight="1">
       <c r="A1" s="3" t="s">
         <v>69</v>
       </c>
@@ -538,8 +597,14 @@
       <c r="F1" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" s="3" t="s">
         <v>70</v>
       </c>
@@ -554,8 +619,10 @@
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="3" t="s">
         <v>70</v>
       </c>
@@ -574,8 +641,14 @@
       <c r="F3" s="1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="G3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="42">
       <c r="A4" s="3" t="s">
         <v>70</v>
       </c>
@@ -594,8 +667,14 @@
       <c r="F4" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="70">
       <c r="A5" s="3" t="s">
         <v>70</v>
       </c>
@@ -614,8 +693,14 @@
       <c r="F5" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6" s="3" t="s">
         <v>70</v>
       </c>
@@ -634,8 +719,14 @@
       <c r="F6" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="28">
       <c r="A7" s="3" t="s">
         <v>70</v>
       </c>
@@ -654,8 +745,14 @@
       <c r="F7" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8" s="3" t="s">
         <v>70</v>
       </c>
@@ -674,8 +771,14 @@
       <c r="F8" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9" s="3" t="s">
         <v>70</v>
       </c>
@@ -690,8 +793,10 @@
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10" s="3" t="s">
         <v>70</v>
       </c>
@@ -708,8 +813,14 @@
       <c r="F10" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="G10" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11" s="3" t="s">
         <v>70</v>
       </c>
@@ -722,8 +833,10 @@
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-    </row>
-    <row r="12" spans="1:6">
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12" s="3" t="s">
         <v>70</v>
       </c>
@@ -736,8 +849,10 @@
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-    </row>
-    <row r="13" spans="1:6">
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" s="3" t="s">
         <v>70</v>
       </c>
@@ -750,8 +865,10 @@
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-    </row>
-    <row r="14" spans="1:6">
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" s="3" t="s">
         <v>70</v>
       </c>
@@ -764,8 +881,10 @@
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6">
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" s="3" t="s">
         <v>70</v>
       </c>
@@ -782,8 +901,14 @@
       <c r="F15" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
+      <c r="G15" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" s="3" t="s">
         <v>70</v>
       </c>
@@ -798,8 +923,10 @@
       </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
-    </row>
-    <row r="17" spans="1:6">
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+    </row>
+    <row r="17" spans="1:8" ht="28">
       <c r="A17" s="3" t="s">
         <v>70</v>
       </c>
@@ -818,8 +945,14 @@
       <c r="F17" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="18" spans="1:6">
+      <c r="G17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="28">
       <c r="A18" s="3" t="s">
         <v>70</v>
       </c>
@@ -838,8 +971,14 @@
       <c r="F18" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="19" spans="1:6">
+      <c r="G18" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" s="3" t="s">
         <v>70</v>
       </c>
@@ -854,8 +993,10 @@
       </c>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
-    </row>
-    <row r="20" spans="1:6">
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" s="3" t="s">
         <v>70</v>
       </c>
@@ -870,8 +1011,10 @@
       </c>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
-    </row>
-    <row r="21" spans="1:6">
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21" s="3" t="s">
         <v>70</v>
       </c>
@@ -886,8 +1029,10 @@
       </c>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
-    </row>
-    <row r="22" spans="1:6">
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22" s="3" t="s">
         <v>70</v>
       </c>
@@ -902,8 +1047,10 @@
       </c>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
-    </row>
-    <row r="23" spans="1:6">
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23" s="3" t="s">
         <v>70</v>
       </c>
@@ -918,8 +1065,10 @@
       </c>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
-    </row>
-    <row r="24" spans="1:6">
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24" s="3" t="s">
         <v>70</v>
       </c>
@@ -936,8 +1085,14 @@
       <c r="F24" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="25" spans="1:6">
+      <c r="G24" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25" s="3" t="s">
         <v>70</v>
       </c>
@@ -952,8 +1107,10 @@
       </c>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
-    </row>
-    <row r="26" spans="1:6">
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26" s="3" t="s">
         <v>70</v>
       </c>
@@ -972,8 +1129,14 @@
       <c r="F26" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
+      <c r="G26" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27" s="3" t="s">
         <v>70</v>
       </c>
@@ -986,8 +1149,14 @@
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
-    </row>
-    <row r="28" spans="1:6">
+      <c r="G27" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="28">
       <c r="A28" s="3" t="s">
         <v>70</v>
       </c>
@@ -1000,8 +1169,14 @@
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
-    </row>
-    <row r="29" spans="1:6">
+      <c r="G28" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29" s="3" t="s">
         <v>70</v>
       </c>
@@ -1014,8 +1189,10 @@
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
-    </row>
-    <row r="30" spans="1:6">
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+    </row>
+    <row r="30" spans="1:8" ht="28">
       <c r="A30" s="3" t="s">
         <v>70</v>
       </c>
@@ -1028,8 +1205,14 @@
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
-    </row>
-    <row r="31" spans="1:6">
+      <c r="G30" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31" s="3" t="s">
         <v>70</v>
       </c>
@@ -1042,8 +1225,10 @@
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
-    </row>
-    <row r="32" spans="1:6">
+      <c r="G31" s="5"/>
+      <c r="H31" s="5"/>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32" s="3" t="s">
         <v>70</v>
       </c>
@@ -1058,8 +1243,10 @@
       </c>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
-    </row>
-    <row r="33" spans="1:6">
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33" s="3" t="s">
         <v>70</v>
       </c>
@@ -1074,8 +1261,10 @@
       </c>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
-    </row>
-    <row r="34" spans="1:6">
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34" s="3" t="s">
         <v>70</v>
       </c>
@@ -1090,8 +1279,10 @@
       </c>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
-    </row>
-    <row r="35" spans="1:6">
+      <c r="G34" s="5"/>
+      <c r="H34" s="5"/>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" s="3" t="s">
         <v>70</v>
       </c>
@@ -1106,8 +1297,10 @@
       </c>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
-    </row>
-    <row r="36" spans="1:6">
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36" s="3" t="s">
         <v>70</v>
       </c>
@@ -1122,8 +1315,10 @@
       </c>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
-    </row>
-    <row r="37" spans="1:6">
+      <c r="G36" s="5"/>
+      <c r="H36" s="5"/>
+    </row>
+    <row r="37" spans="1:8" ht="28">
       <c r="A37" s="3" t="s">
         <v>70</v>
       </c>
@@ -1142,8 +1337,14 @@
       <c r="F37" s="1" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="38" spans="1:6">
+      <c r="G37" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="28">
       <c r="A38" s="3" t="s">
         <v>70</v>
       </c>
@@ -1162,8 +1363,14 @@
       <c r="F38" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="39" spans="1:6">
+      <c r="G38" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39" s="3" t="s">
         <v>70</v>
       </c>
@@ -1178,8 +1385,10 @@
       </c>
       <c r="E39" s="1"/>
       <c r="F39" s="1"/>
-    </row>
-    <row r="40" spans="1:6">
+      <c r="G39" s="5"/>
+      <c r="H39" s="5"/>
+    </row>
+    <row r="40" spans="1:8" ht="42">
       <c r="A40" s="3" t="s">
         <v>70</v>
       </c>
@@ -1194,8 +1403,14 @@
       </c>
       <c r="E40" s="1"/>
       <c r="F40" s="1"/>
-    </row>
-    <row r="41" spans="1:6">
+      <c r="G40" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="56">
       <c r="A41" s="3" t="s">
         <v>70</v>
       </c>
@@ -1210,8 +1425,14 @@
       </c>
       <c r="E41" s="1"/>
       <c r="F41" s="1"/>
-    </row>
-    <row r="42" spans="1:6">
+      <c r="G41" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H41" s="5" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" s="3" t="s">
         <v>70</v>
       </c>
@@ -1226,8 +1447,10 @@
       </c>
       <c r="E42" s="1"/>
       <c r="F42" s="1"/>
-    </row>
-    <row r="43" spans="1:6">
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+    </row>
+    <row r="43" spans="1:8" ht="42">
       <c r="A43" s="3" t="s">
         <v>70</v>
       </c>
@@ -1246,8 +1469,14 @@
       <c r="F43" s="1" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="44" spans="1:6">
+      <c r="G43" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44" s="3" t="s">
         <v>70</v>
       </c>
@@ -1265,6 +1494,12 @@
       </c>
       <c r="F44" s="1" t="s">
         <v>20</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H44" s="5" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(PDG-63): align media SourceType and attachment types with picklist
- PCIJ_CORRUPTION_WATCH / PCIJ_INVESTIGATIVE_REPORTS: SourceType "Media"
  (independent newsroom, not a government body); add Media to the
  Sources.SourceType picklist and describe both values.
- Attachments.Type: use the picklist's Image instead of Photograph (PCIJ,
  DTI) and "IMAGE"; use Document instead of "PDF" (AMLC).
- Picklist: add PCIJ_INVESTIGATIVE_REPORTS / DTI_FAIR_TRADE_PRESS_RELEASES
  dataset names and the DTI source name.
- Golden test expects Media and Image accordingly.
</commit_message>
<xml_diff>
--- a/data/rules/mediaMapping.xlsx
+++ b/data/rules/mediaMapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30992BEC-44E3-4C62-A676-9A8A06396926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FDDF245-AD07-4732-B12E-38C3E5583B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="141">
   <si>
     <t>Entity Category</t>
   </si>
@@ -283,9 +283,6 @@
     <t>constant*constant*constant</t>
   </si>
   <si>
-    <t>"IMAGE"*"IMAGE"*"PDF"</t>
-  </si>
-  <si>
     <t>Attachments[].URL</t>
   </si>
   <si>
@@ -391,9 +388,6 @@
     <t>constant*constant*constant*constant*constant*constant</t>
   </si>
   <si>
-    <t>"Table"*"Chart"*"Dashboard"*"Document"*"Photograph"*"Document"</t>
-  </si>
-  <si>
     <t>list_expand*list_expand*list_expand*list_expand*list_expand*list_expand</t>
   </si>
   <si>
@@ -442,10 +436,13 @@
     <t>"Department of Trade and Industry (Philippines)"</t>
   </si>
   <si>
-    <t>"Photograph"*"Photograph"*"Document"</t>
+    <t>_embedded.wp:term[].name</t>
   </si>
   <si>
-    <t>_embedded.wp:term[].name</t>
+    <t>"Image"*"Image"*"Document"</t>
+  </si>
+  <si>
+    <t>"Table"*"Chart"*"Dashboard"*"Document"*"Image"*"Document"</t>
   </si>
 </sst>
 </file>
@@ -827,28 +824,28 @@
         <v>9</v>
       </c>
       <c r="K1" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="L1" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="L1" s="5" t="s">
-        <v>97</v>
-      </c>
       <c r="M1" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="N1" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="N1" s="5" t="s">
-        <v>103</v>
-      </c>
       <c r="O1" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="P1" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="P1" s="12" t="s">
-        <v>118</v>
-      </c>
       <c r="Q1" s="12" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="R1" s="12" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="S1" s="8"/>
       <c r="T1" s="8"/>
@@ -922,7 +919,7 @@
         <v>16</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K3" s="10" t="s">
         <v>16</v>
@@ -940,7 +937,7 @@
         <v>16</v>
       </c>
       <c r="P3" s="9" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="Q3" s="9" t="s">
         <v>16</v>
@@ -973,13 +970,13 @@
         <v>16</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>16</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="I4" s="9" t="s">
         <v>16</v>
@@ -991,7 +988,7 @@
         <v>16</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M4" s="9" t="s">
         <v>16</v>
@@ -1009,7 +1006,7 @@
         <v>16</v>
       </c>
       <c r="R4" s="9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="S4" s="8"/>
       <c r="T4" s="8"/>
@@ -1054,25 +1051,25 @@
         <v>16</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M5" s="9" t="s">
         <v>16</v>
       </c>
       <c r="N5" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="O5" s="9" t="s">
         <v>16</v>
       </c>
       <c r="P5" s="9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Q5" s="9" t="s">
         <v>16</v>
       </c>
       <c r="R5" s="9" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="S5" s="8"/>
       <c r="T5" s="8"/>
@@ -1117,13 +1114,13 @@
         <v>16</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M6" s="9" t="s">
         <v>16</v>
       </c>
       <c r="N6" s="9" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O6" s="9" t="s">
         <v>16</v>
@@ -1135,7 +1132,7 @@
         <v>16</v>
       </c>
       <c r="R6" s="9" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="S6" s="8"/>
       <c r="T6" s="8"/>
@@ -1198,7 +1195,7 @@
         <v>29</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
@@ -1249,7 +1246,7 @@
         <v>29</v>
       </c>
       <c r="N8" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O8" s="9" t="s">
         <v>29</v>
@@ -1357,7 +1354,7 @@
         <v>29</v>
       </c>
       <c r="R10" s="9" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="S10" s="8"/>
       <c r="T10" s="8"/>
@@ -1421,13 +1418,13 @@
         <v>29</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M12" s="9" t="s">
         <v>29</v>
       </c>
       <c r="N12" s="9" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O12" s="8"/>
       <c r="P12" s="8"/>
@@ -1540,13 +1537,13 @@
         <v>29</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M15" s="9" t="s">
         <v>29</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>29</v>
@@ -1558,7 +1555,7 @@
         <v>29</v>
       </c>
       <c r="R15" s="9" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="S15" s="8"/>
       <c r="T15" s="8"/>
@@ -1674,10 +1671,10 @@
         <v>49</v>
       </c>
       <c r="M18" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="N18" s="9" t="s">
         <v>109</v>
-      </c>
-      <c r="N18" s="9" t="s">
-        <v>110</v>
       </c>
       <c r="O18" s="9" t="s">
         <v>16</v>
@@ -1686,10 +1683,10 @@
         <v>49</v>
       </c>
       <c r="Q18" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="R18" s="11" t="s">
         <v>109</v>
-      </c>
-      <c r="R18" s="11" t="s">
-        <v>110</v>
       </c>
       <c r="S18" s="8"/>
       <c r="T18" s="8"/>
@@ -1737,10 +1734,10 @@
         <v>51</v>
       </c>
       <c r="M19" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="N19" s="9" t="s">
         <v>111</v>
-      </c>
-      <c r="N19" s="9" t="s">
-        <v>112</v>
       </c>
       <c r="O19" s="9" t="s">
         <v>29</v>
@@ -1749,10 +1746,10 @@
         <v>51</v>
       </c>
       <c r="Q19" s="11" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="R19" s="11" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="S19" s="8"/>
       <c r="T19" s="8"/>
@@ -1970,13 +1967,13 @@
         <v>16</v>
       </c>
       <c r="L25" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="M25" s="9" t="s">
         <v>29</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="O25" s="9" t="s">
         <v>16</v>
@@ -1988,7 +1985,7 @@
         <v>16</v>
       </c>
       <c r="R25" s="9" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="S25" s="8"/>
       <c r="T25" s="8"/>
@@ -2078,7 +2075,7 @@
         <v>29</v>
       </c>
       <c r="R27" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="S27" s="8"/>
       <c r="T27" s="8"/>
@@ -2156,7 +2153,7 @@
         <v>67</v>
       </c>
       <c r="R29" s="11" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="S29" s="8"/>
       <c r="T29" s="8"/>
@@ -2185,7 +2182,7 @@
         <v>67</v>
       </c>
       <c r="J30" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8"/>
@@ -2195,7 +2192,7 @@
         <v>67</v>
       </c>
       <c r="P30" s="9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="Q30" s="8"/>
       <c r="R30" s="8"/>
@@ -2490,10 +2487,10 @@
         <v>81</v>
       </c>
       <c r="M38" s="9" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N38" s="9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="O38" s="9" t="s">
         <v>16</v>
@@ -2553,10 +2550,10 @@
         <v>30</v>
       </c>
       <c r="M39" s="9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="O39" s="9" t="s">
         <v>29</v>
@@ -2568,7 +2565,7 @@
         <v>29</v>
       </c>
       <c r="R39" s="9" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="S39" s="8"/>
       <c r="T39" s="8"/>
@@ -2613,7 +2610,7 @@
       <c r="X40" s="8"/>
       <c r="Y40" s="8"/>
     </row>
-    <row r="41" spans="1:25" ht="89" thickBot="1">
+    <row r="41" spans="1:25" ht="76.5" thickBot="1">
       <c r="A41" s="3" t="s">
         <v>10</v>
       </c>
@@ -2632,29 +2629,29 @@
         <v>86</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>87</v>
+        <v>139</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J41" s="9" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="K41" s="8"/>
       <c r="L41" s="8"/>
       <c r="M41" s="8"/>
       <c r="N41" s="8"/>
       <c r="O41" s="9" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="Q41" s="9" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="R41" s="11" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="S41" s="8"/>
       <c r="T41" s="8"/>
@@ -2669,7 +2666,7 @@
         <v>10</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>15</v>
@@ -2680,32 +2677,32 @@
       <c r="E42" s="7"/>
       <c r="F42" s="7"/>
       <c r="G42" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H42" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H42" s="3" t="s">
-        <v>90</v>
-      </c>
       <c r="I42" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="J42" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
       <c r="M42" s="8"/>
       <c r="N42" s="8"/>
       <c r="O42" s="9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="P42" s="9" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="Q42" s="9" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="R42" s="9" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="S42" s="8"/>
       <c r="T42" s="8"/>
@@ -2720,13 +2717,13 @@
         <v>10</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E43" s="7"/>
       <c r="F43" s="7"/>
@@ -2755,25 +2752,25 @@
         <v>10</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E44" s="9" t="s">
         <v>16</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>16</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I44" s="8"/>
       <c r="J44" s="8"/>
@@ -2781,13 +2778,13 @@
         <v>16</v>
       </c>
       <c r="L44" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M44" s="9" t="s">
         <v>16</v>
       </c>
       <c r="N44" s="9" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="O44" s="8"/>
       <c r="P44" s="8"/>
@@ -2806,13 +2803,13 @@
         <v>10</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>29</v>
@@ -2838,7 +2835,7 @@
         <v>29</v>
       </c>
       <c r="N45" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="O45" s="8"/>
       <c r="P45" s="8"/>

</xml_diff>

<commit_message>
refactor(PDG-65): rename DTI source and dataset to DTI_PH
"DTI" is not unique across countries, so follow the country-suffixed naming
of DOJ_PH / SEC_PH: source_name DTI -> DTI_PH and dataset
DTI_FAIR_TRADE_PRESS_RELEASES -> DTI_PH_FAIR_TRADE_PRESS_RELEASES across
mediaSources.yaml, mediaMapping/mediaPickLists/mediaPreNormalization, the
golden test and its fixture file.

mediaMapping.xlsx is binary, so this commit also carries two unrelated mapping
edits made in the same file: the Taxonomy.* rows renamed to Metadata.*, and
DOJ_PH_NEWS Publisher.Name set to "Department of Justice (Philippines)".

Existing environments need common.lkup_media_source / lkup_media_dataset rows
named DTI_PH / DTI_PH_FAIR_TRADE_PRESS_RELEASES.
</commit_message>
<xml_diff>
--- a/data/rules/mediaMapping.xlsx
+++ b/data/rules/mediaMapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FDDF245-AD07-4732-B12E-38C3E5583B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{982AEC87-1FF8-4581-A866-039754EA62D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="142">
   <si>
     <t>Entity Category</t>
   </si>
@@ -214,13 +214,7 @@
     <t>author</t>
   </si>
   <si>
-    <t>Taxonomy.Language</t>
-  </si>
-  <si>
     <t>"en"</t>
-  </si>
-  <si>
-    <t>Taxonomy.Categories[]</t>
   </si>
   <si>
     <t>list_expand</t>
@@ -229,16 +223,7 @@
     <t>category</t>
   </si>
   <si>
-    <t>Taxonomy.Tags[]</t>
-  </si>
-  <si>
-    <t>Taxonomy.Topics[]</t>
-  </si>
-  <si>
     <t>type</t>
-  </si>
-  <si>
-    <t>Taxonomy.Keywords[]</t>
   </si>
   <si>
     <t>Locations[]</t>
@@ -394,19 +379,7 @@
     <t>TableEmbedUrls*ChartEmbedUrls*DashboardEmbedUrls*DocumentUrls*FeaturedImageUrl*EmbeddedPdfUrls</t>
   </si>
   <si>
-    <t>DTI_FAIR_TRADE_PRESS_RELEASES TYPE</t>
-  </si>
-  <si>
-    <t>DTI_FAIR_TRADE_PRESS_RELEASES</t>
-  </si>
-  <si>
     <t>"Media"</t>
-  </si>
-  <si>
-    <t>"DTI_FAIR_TRADE_PRESS_RELEASES"</t>
-  </si>
-  <si>
-    <t>"DTI"</t>
   </si>
   <si>
     <t>link</t>
@@ -443,6 +416,36 @@
   </si>
   <si>
     <t>"Table"*"Chart"*"Dashboard"*"Document"*"Image"*"Document"</t>
+  </si>
+  <si>
+    <t>Metadata.Language</t>
+  </si>
+  <si>
+    <t>Metadata.Categories[]</t>
+  </si>
+  <si>
+    <t>Metadata.Tags[]</t>
+  </si>
+  <si>
+    <t>Metadata.Topics[]</t>
+  </si>
+  <si>
+    <t>Metadata.Keywords[]</t>
+  </si>
+  <si>
+    <t>DTI_PH_FAIR_TRADE_PRESS_RELEASES TYPE</t>
+  </si>
+  <si>
+    <t>DTI_PH_FAIR_TRADE_PRESS_RELEASES</t>
+  </si>
+  <si>
+    <t>"DTI_PH_FAIR_TRADE_PRESS_RELEASES"</t>
+  </si>
+  <si>
+    <t>"DTI_PH"</t>
+  </si>
+  <si>
+    <t>"Department of Justice (Philippines)"</t>
   </si>
 </sst>
 </file>
@@ -824,28 +827,28 @@
         <v>9</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="L1" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="M1" s="5" t="s">
-        <v>101</v>
-      </c>
       <c r="N1" s="5" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="O1" s="12" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="P1" s="12" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="Q1" s="12" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="R1" s="12" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="S1" s="8"/>
       <c r="T1" s="8"/>
@@ -919,7 +922,7 @@
         <v>16</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="K3" s="10" t="s">
         <v>16</v>
@@ -937,7 +940,7 @@
         <v>16</v>
       </c>
       <c r="P3" s="9" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="Q3" s="9" t="s">
         <v>16</v>
@@ -970,13 +973,13 @@
         <v>16</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>16</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="I4" s="9" t="s">
         <v>16</v>
@@ -988,7 +991,7 @@
         <v>16</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="M4" s="9" t="s">
         <v>16</v>
@@ -1006,7 +1009,7 @@
         <v>16</v>
       </c>
       <c r="R4" s="9" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="S4" s="8"/>
       <c r="T4" s="8"/>
@@ -1051,25 +1054,25 @@
         <v>16</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="M5" s="9" t="s">
         <v>16</v>
       </c>
       <c r="N5" s="9" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="O5" s="9" t="s">
         <v>16</v>
       </c>
       <c r="P5" s="9" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="Q5" s="9" t="s">
         <v>16</v>
       </c>
       <c r="R5" s="9" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="S5" s="8"/>
       <c r="T5" s="8"/>
@@ -1114,13 +1117,13 @@
         <v>16</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="M6" s="9" t="s">
         <v>16</v>
       </c>
       <c r="N6" s="9" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="O6" s="9" t="s">
         <v>16</v>
@@ -1132,7 +1135,7 @@
         <v>16</v>
       </c>
       <c r="R6" s="9" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="S6" s="8"/>
       <c r="T6" s="8"/>
@@ -1195,7 +1198,7 @@
         <v>29</v>
       </c>
       <c r="R7" s="9" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
@@ -1246,7 +1249,7 @@
         <v>29</v>
       </c>
       <c r="N8" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="O8" s="9" t="s">
         <v>29</v>
@@ -1354,7 +1357,7 @@
         <v>29</v>
       </c>
       <c r="R10" s="9" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="S10" s="8"/>
       <c r="T10" s="8"/>
@@ -1418,13 +1421,13 @@
         <v>29</v>
       </c>
       <c r="L12" s="10" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="M12" s="9" t="s">
         <v>29</v>
       </c>
       <c r="N12" s="9" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="O12" s="8"/>
       <c r="P12" s="8"/>
@@ -1537,13 +1540,13 @@
         <v>29</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="M15" s="9" t="s">
         <v>29</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>29</v>
@@ -1555,7 +1558,7 @@
         <v>29</v>
       </c>
       <c r="R15" s="9" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="S15" s="8"/>
       <c r="T15" s="8"/>
@@ -1671,10 +1674,10 @@
         <v>49</v>
       </c>
       <c r="M18" s="9" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="N18" s="9" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="O18" s="9" t="s">
         <v>16</v>
@@ -1683,10 +1686,10 @@
         <v>49</v>
       </c>
       <c r="Q18" s="11" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="R18" s="11" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="S18" s="8"/>
       <c r="T18" s="8"/>
@@ -1734,10 +1737,10 @@
         <v>51</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="O19" s="9" t="s">
         <v>29</v>
@@ -1746,10 +1749,10 @@
         <v>51</v>
       </c>
       <c r="Q19" s="11" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="R19" s="11" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="S19" s="8"/>
       <c r="T19" s="8"/>
@@ -1934,7 +1937,7 @@
       <c r="X24" s="8"/>
       <c r="Y24" s="8"/>
     </row>
-    <row r="25" spans="1:25" ht="26.5" thickBot="1">
+    <row r="25" spans="1:25" ht="29" thickBot="1">
       <c r="A25" s="3" t="s">
         <v>10</v>
       </c>
@@ -1967,13 +1970,13 @@
         <v>16</v>
       </c>
       <c r="L25" s="10" t="s">
-        <v>98</v>
+        <v>141</v>
       </c>
       <c r="M25" s="9" t="s">
         <v>29</v>
       </c>
       <c r="N25" s="9" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="O25" s="9" t="s">
         <v>16</v>
@@ -1985,7 +1988,7 @@
         <v>16</v>
       </c>
       <c r="R25" s="9" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="S25" s="8"/>
       <c r="T25" s="8"/>
@@ -2075,7 +2078,7 @@
         <v>29</v>
       </c>
       <c r="R27" s="9" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="S27" s="8"/>
       <c r="T27" s="8"/>
@@ -2090,7 +2093,7 @@
         <v>10</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>64</v>
+        <v>132</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>15</v>
@@ -2102,7 +2105,7 @@
         <v>16</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I28" s="8"/>
       <c r="J28" s="8"/>
@@ -2127,7 +2130,7 @@
         <v>10</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>66</v>
+        <v>133</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>12</v>
@@ -2136,10 +2139,10 @@
       <c r="E29" s="7"/>
       <c r="F29" s="7"/>
       <c r="G29" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I29" s="8"/>
       <c r="J29" s="8"/>
@@ -2150,10 +2153,10 @@
       <c r="O29" s="8"/>
       <c r="P29" s="8"/>
       <c r="Q29" s="11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="R29" s="11" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="S29" s="8"/>
       <c r="T29" s="8"/>
@@ -2168,7 +2171,7 @@
         <v>10</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>69</v>
+        <v>134</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>12</v>
@@ -2179,20 +2182,20 @@
       <c r="G30" s="8"/>
       <c r="H30" s="8"/>
       <c r="I30" s="9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="J30" s="9" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8"/>
       <c r="M30" s="8"/>
       <c r="N30" s="8"/>
       <c r="O30" s="9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="P30" s="9" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="Q30" s="8"/>
       <c r="R30" s="8"/>
@@ -2209,7 +2212,7 @@
         <v>10</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>70</v>
+        <v>135</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>12</v>
@@ -2218,10 +2221,10 @@
       <c r="E31" s="7"/>
       <c r="F31" s="7"/>
       <c r="G31" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="H31" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="I31" s="8"/>
       <c r="J31" s="8"/>
@@ -2246,7 +2249,7 @@
         <v>10</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>72</v>
+        <v>136</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>12</v>
@@ -2279,13 +2282,13 @@
         <v>10</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
@@ -2314,13 +2317,13 @@
         <v>10</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E34" s="7"/>
       <c r="F34" s="7"/>
@@ -2349,13 +2352,13 @@
         <v>10</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E35" s="7"/>
       <c r="F35" s="7"/>
@@ -2384,13 +2387,13 @@
         <v>10</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
@@ -2419,13 +2422,13 @@
         <v>10</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E37" s="7"/>
       <c r="F37" s="7"/>
@@ -2454,55 +2457,55 @@
         <v>10</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E38" s="9" t="s">
         <v>16</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="G38" s="9" t="s">
         <v>16</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="I38" s="9" t="s">
         <v>16</v>
       </c>
       <c r="J38" s="9" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="K38" s="10" t="s">
         <v>16</v>
       </c>
       <c r="L38" s="10" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="M38" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="N38" s="9" t="s">
         <v>108</v>
-      </c>
-      <c r="N38" s="9" t="s">
-        <v>113</v>
       </c>
       <c r="O38" s="9" t="s">
         <v>16</v>
       </c>
       <c r="P38" s="9" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="Q38" s="9" t="s">
         <v>16</v>
       </c>
       <c r="R38" s="9" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="S38" s="8"/>
       <c r="T38" s="8"/>
@@ -2517,13 +2520,13 @@
         <v>10</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>29</v>
@@ -2550,10 +2553,10 @@
         <v>30</v>
       </c>
       <c r="M39" s="9" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="O39" s="9" t="s">
         <v>29</v>
@@ -2565,7 +2568,7 @@
         <v>29</v>
       </c>
       <c r="R39" s="9" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
       <c r="S39" s="8"/>
       <c r="T39" s="8"/>
@@ -2580,13 +2583,13 @@
         <v>10</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E40" s="7"/>
       <c r="F40" s="7"/>
@@ -2615,43 +2618,43 @@
         <v>10</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E41" s="7"/>
       <c r="F41" s="7"/>
       <c r="G41" s="3" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="J41" s="9" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="K41" s="8"/>
       <c r="L41" s="8"/>
       <c r="M41" s="8"/>
       <c r="N41" s="8"/>
       <c r="O41" s="9" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="Q41" s="9" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="R41" s="11" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="S41" s="8"/>
       <c r="T41" s="8"/>
@@ -2666,43 +2669,43 @@
         <v>10</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="E42" s="7"/>
       <c r="F42" s="7"/>
       <c r="G42" s="3" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="I42" s="9" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="J42" s="9" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
       <c r="M42" s="8"/>
       <c r="N42" s="8"/>
       <c r="O42" s="9" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="P42" s="9" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="Q42" s="9" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="R42" s="9" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="S42" s="8"/>
       <c r="T42" s="8"/>
@@ -2717,13 +2720,13 @@
         <v>10</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E43" s="7"/>
       <c r="F43" s="7"/>
@@ -2752,25 +2755,25 @@
         <v>10</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E44" s="9" t="s">
         <v>16</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="G44" s="9" t="s">
         <v>16</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="I44" s="8"/>
       <c r="J44" s="8"/>
@@ -2778,13 +2781,13 @@
         <v>16</v>
       </c>
       <c r="L44" s="10" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="M44" s="9" t="s">
         <v>16</v>
       </c>
       <c r="N44" s="9" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="O44" s="8"/>
       <c r="P44" s="8"/>
@@ -2803,13 +2806,13 @@
         <v>10</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>29</v>
@@ -2835,7 +2838,7 @@
         <v>29</v>
       </c>
       <c r="N45" s="9" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="O45" s="8"/>
       <c r="P45" s="8"/>

</xml_diff>

<commit_message>
feat(PDG-71): add PTV_NEWS media source
Collect Local News, Provincial News and Business articles from the PTV WordPress API, with the reporter byline as author, the featured image as thumbnail, and in-article images and documents as attachments.
</commit_message>
<xml_diff>
--- a/data/rules/mediaMapping.xlsx
+++ b/data/rules/mediaMapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cloned repos\python-components\data\rules\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{923DB59D-25CB-4493-B5C3-34DB0D3BCC30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572D1EA0-B232-4613-993A-461E4A579B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="169">
   <si>
     <t>Entity Category</t>
   </si>
@@ -504,6 +504,30 @@
   <si>
     <t>EntityType</t>
   </si>
+  <si>
+    <t>PTV_NEWS TYPE</t>
+  </si>
+  <si>
+    <t>PTV_NEWS</t>
+  </si>
+  <si>
+    <t>"PTV_NEWS"</t>
+  </si>
+  <si>
+    <t>"PTV"</t>
+  </si>
+  <si>
+    <t>"People's Television Network (Philippines)"</t>
+  </si>
+  <si>
+    <t>Author</t>
+  </si>
+  <si>
+    <t>_embedded.wp:featuredmedia[].source_url*ImageUrls*DocumentUrls</t>
+  </si>
+  <si>
+    <t>"Thumbnail"*"Image"*"Document"</t>
+  </si>
 </sst>
 </file>
 
@@ -929,8 +953,12 @@
       <c r="V1" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="W1" s="8"/>
-      <c r="X1" s="8"/>
+      <c r="W1" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="X1" s="13" t="s">
+        <v>162</v>
+      </c>
       <c r="Y1" s="8"/>
       <c r="Z1" s="8"/>
       <c r="AA1" s="8"/>
@@ -1043,8 +1071,12 @@
       <c r="V3" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="W3" s="8"/>
-      <c r="X3" s="8"/>
+      <c r="W3" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="X3" s="9" t="s">
+        <v>17</v>
+      </c>
       <c r="Y3" s="8"/>
       <c r="Z3" s="8"/>
       <c r="AA3" s="8"/>
@@ -1118,8 +1150,12 @@
       <c r="V4" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="W4" s="8"/>
-      <c r="X4" s="8"/>
+      <c r="W4" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="X4" s="9" t="s">
+        <v>19</v>
+      </c>
       <c r="Y4" s="8"/>
       <c r="Z4" s="8"/>
       <c r="AA4" s="8"/>
@@ -1193,8 +1229,12 @@
       <c r="V5" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="W5" s="8"/>
-      <c r="X5" s="8"/>
+      <c r="W5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="X5" s="9" t="s">
+        <v>163</v>
+      </c>
       <c r="Y5" s="8"/>
       <c r="Z5" s="8"/>
       <c r="AA5" s="8"/>
@@ -1268,8 +1308,12 @@
       <c r="V6" s="11" t="s">
         <v>154</v>
       </c>
-      <c r="W6" s="8"/>
-      <c r="X6" s="8"/>
+      <c r="W6" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="X6" s="9" t="s">
+        <v>164</v>
+      </c>
       <c r="Y6" s="8"/>
       <c r="Z6" s="8"/>
       <c r="AA6" s="8"/>
@@ -1343,8 +1387,12 @@
       <c r="V7" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="W7" s="8"/>
-      <c r="X7" s="8"/>
+      <c r="W7" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="X7" s="9" t="s">
+        <v>120</v>
+      </c>
       <c r="Y7" s="8"/>
       <c r="Z7" s="8"/>
       <c r="AA7" s="8"/>
@@ -1418,8 +1466,12 @@
       <c r="V8" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="W8" s="8"/>
-      <c r="X8" s="8"/>
+      <c r="W8" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="X8" s="9" t="s">
+        <v>33</v>
+      </c>
       <c r="Y8" s="8"/>
       <c r="Z8" s="8"/>
       <c r="AA8" s="8"/>
@@ -1465,7 +1517,7 @@
       <c r="AB9" s="8"/>
       <c r="AC9" s="8"/>
     </row>
-    <row r="10" spans="1:29" ht="15" thickBot="1">
+    <row r="10" spans="1:29" ht="26.5" thickBot="1">
       <c r="A10" s="3" t="s">
         <v>10</v>
       </c>
@@ -1526,8 +1578,12 @@
       </c>
       <c r="U10" s="8"/>
       <c r="V10" s="8"/>
-      <c r="W10" s="8"/>
-      <c r="X10" s="8"/>
+      <c r="W10" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="X10" s="9" t="s">
+        <v>121</v>
+      </c>
       <c r="Y10" s="8"/>
       <c r="Z10" s="8"/>
       <c r="AA10" s="8"/>
@@ -1755,8 +1811,12 @@
       <c r="V15" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="W15" s="8"/>
-      <c r="X15" s="8"/>
+      <c r="W15" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="X15" s="9" t="s">
+        <v>122</v>
+      </c>
       <c r="Y15" s="8"/>
       <c r="Z15" s="8"/>
       <c r="AA15" s="8"/>
@@ -1906,8 +1966,12 @@
       <c r="V18" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="W18" s="8"/>
-      <c r="X18" s="8"/>
+      <c r="W18" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="X18" s="9" t="s">
+        <v>104</v>
+      </c>
       <c r="Y18" s="8"/>
       <c r="Z18" s="8"/>
       <c r="AA18" s="8"/>
@@ -1981,8 +2045,12 @@
       <c r="V19" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="W19" s="8"/>
-      <c r="X19" s="8"/>
+      <c r="W19" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="X19" s="9" t="s">
+        <v>127</v>
+      </c>
       <c r="Y19" s="8"/>
       <c r="Z19" s="8"/>
       <c r="AA19" s="8"/>
@@ -2249,8 +2317,12 @@
       <c r="V25" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="W25" s="8"/>
-      <c r="X25" s="8"/>
+      <c r="W25" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="X25" s="9" t="s">
+        <v>165</v>
+      </c>
       <c r="Y25" s="8"/>
       <c r="Z25" s="8"/>
       <c r="AA25" s="8"/>
@@ -2351,8 +2423,12 @@
       </c>
       <c r="U27" s="8"/>
       <c r="V27" s="8"/>
-      <c r="W27" s="8"/>
-      <c r="X27" s="8"/>
+      <c r="W27" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="X27" s="9" t="s">
+        <v>166</v>
+      </c>
       <c r="Y27" s="8"/>
       <c r="Z27" s="8"/>
       <c r="AA27" s="8"/>
@@ -2453,7 +2529,7 @@
       <c r="AB29" s="8"/>
       <c r="AC29" s="8"/>
     </row>
-    <row r="30" spans="1:29" ht="29.5" thickBot="1">
+    <row r="30" spans="1:29" ht="39" thickBot="1">
       <c r="A30" s="3" t="s">
         <v>10</v>
       </c>
@@ -2494,8 +2570,12 @@
       <c r="V30" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="W30" s="8"/>
-      <c r="X30" s="8"/>
+      <c r="W30" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="X30" s="9" t="s">
+        <v>129</v>
+      </c>
       <c r="Y30" s="8"/>
       <c r="Z30" s="8"/>
       <c r="AA30" s="8"/>
@@ -2842,8 +2922,12 @@
       <c r="V38" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="W38" s="8"/>
-      <c r="X38" s="8"/>
+      <c r="W38" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="X38" s="9" t="s">
+        <v>76</v>
+      </c>
       <c r="Y38" s="8"/>
       <c r="Z38" s="8"/>
       <c r="AA38" s="8"/>
@@ -2917,8 +3001,12 @@
       <c r="V39" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="W39" s="8"/>
-      <c r="X39" s="8"/>
+      <c r="W39" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="X39" s="9" t="s">
+        <v>120</v>
+      </c>
       <c r="Y39" s="8"/>
       <c r="Z39" s="8"/>
       <c r="AA39" s="8"/>
@@ -3015,8 +3103,12 @@
       </c>
       <c r="U41" s="8"/>
       <c r="V41" s="8"/>
-      <c r="W41" s="8"/>
-      <c r="X41" s="8"/>
+      <c r="W41" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="X41" s="9" t="s">
+        <v>168</v>
+      </c>
       <c r="Y41" s="8"/>
       <c r="Z41" s="8"/>
       <c r="AA41" s="8"/>
@@ -3074,8 +3166,12 @@
       </c>
       <c r="U42" s="8"/>
       <c r="V42" s="8"/>
-      <c r="W42" s="8"/>
-      <c r="X42" s="8"/>
+      <c r="W42" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="X42" s="9" t="s">
+        <v>167</v>
+      </c>
       <c r="Y42" s="8"/>
       <c r="Z42" s="8"/>
       <c r="AA42" s="8"/>

</xml_diff>